<commit_message>
cambio en graficos SportData_muestra_ejercicioAmazon3.xlsx
</commit_message>
<xml_diff>
--- a/estadistica-excel/SportData_muestra_ejercicioAmazon3.xlsx
+++ b/estadistica-excel/SportData_muestra_ejercicioAmazon3.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -490,6 +490,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -503,9 +506,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -13151,30 +13151,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="12" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="13" t="s">
+      <c r="D1" s="13"/>
+      <c r="E1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="14" t="s">
+      <c r="F1" s="14"/>
+      <c r="G1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="15" t="s">
+      <c r="H1" s="15"/>
+      <c r="I1" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="16" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="16"/>
+      <c r="L1" s="11"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">

</xml_diff>

<commit_message>
actualizo nombre de grafico graficos con todos los valores de producto todo OK
</commit_message>
<xml_diff>
--- a/estadistica-excel/SportData_muestra_ejercicioAmazon3.xlsx
+++ b/estadistica-excel/SportData_muestra_ejercicioAmazon3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\curso_big_data_pauladejuan\nueva_carpeta_repositorio_local\rombo_python_bucles\estadistica-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDABDB4A-0FF0-4CA6-94BA-006D9BA6B973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4905821E-3640-4AD3-A516-00950FFA82E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1564,6 +1564,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Accesorios</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>

</xml_diff>